<commit_message>
Add OCR image preprocessing and ocrmypdf fast-path, add Poppler to waiver
- Preprocessing: grayscale, auto-contrast, sharpen, binarize before Tesseract
- ocrmypdf integration: tries whole-PDF OCR first, falls back to page-by-page
- Tesseract config: LSTM engine + auto page segmentation
- Image parser gets same preprocessing pipeline
- Poppler added to GREEN waiver list (external binary #37)
- All configurable via env vars, zero new pip deps
</commit_message>
<xml_diff>
--- a/docs/05_security/waiver_cheat_sheet_v5.xlsx
+++ b/docs/05_security/waiver_cheat_sheet_v5.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="GREEN - Approved" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="YELLOW - Applying" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="BLUE - Recommended" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="RED - Banned" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RETIRED" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GREEN - Approved" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YELLOW - Applying" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BLUE - Recommended" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RED - Banned" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RETIRED" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -644,7 +644,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>36 (35 pip + 1 binary)</t>
+          <t>37 (35 pip + 2 binaries)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1162,7 +1162,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GREEN -- Approved and Installed (36 direct: 35 pip + 1 binary)</t>
+          <t>GREEN -- Approved and Installed (37 direct: 35 pip + 2 binaries)</t>
         </is>
       </c>
     </row>
@@ -2833,790 +2833,835 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Poppler</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>24.x</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>GPL-2.0</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>freedesktop.org / International OSS</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>External Binary / PDF</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>PDF page rendering engine (pdf2image calls this binary)</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Renders PDF pages to images for OCR pipeline. Required by pdf2image (#17). Used by LibreOffice, GIMP, and most Linux PDF viewers. Installed via winget. Zero network activity.</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>No known CVEs</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Transitive Dependencies (auto-installed, no separate waiver needed)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>Package</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>Pulled In By</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
+    <row r="45">
+      <c r="A45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>annotated-types</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>0.7.0</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>pydantic</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>Type annotation support</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="13" t="n">
+    <row r="46">
+      <c r="A46" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>anyio</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>4.12.1</t>
         </is>
       </c>
-      <c r="D45" s="13" t="inlineStr">
+      <c r="D46" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>httpx</t>
         </is>
       </c>
-      <c r="F45" s="13" t="inlineStr">
+      <c r="F46" s="13" t="inlineStr">
         <is>
           <t>Async I/O abstraction</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
+    <row r="47">
+      <c r="A47" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>cffi</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>2.0.0</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>cryptography</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>C FFI for OpenSSL bindings</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="13" t="n">
+    <row r="48">
+      <c r="A48" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>chardet</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>5.2.0</t>
         </is>
       </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>LGPL-2.1</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E48" s="13" t="inlineStr">
         <is>
           <t>pdfminer.six</t>
         </is>
       </c>
-      <c r="F47" s="13" t="inlineStr">
+      <c r="F48" s="13" t="inlineStr">
         <is>
           <t>Character encoding detection</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+    <row r="49">
+      <c r="A49" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>charset-normalizer</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>3.4.4</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>requests</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>Encoding normalization</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="13" t="n">
+    <row r="50">
+      <c r="A50" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>distro</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C50" s="13" t="inlineStr">
         <is>
           <t>1.9.0</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D50" s="13" t="inlineStr">
         <is>
           <t>Apache 2.0</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>openai</t>
         </is>
       </c>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="F50" s="13" t="inlineStr">
         <is>
           <t>Linux distro detection</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
+    <row r="51">
+      <c r="A51" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>et_xmlfile</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>2.0.0</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>openpyxl</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>XML utility for Excel</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="13" t="n">
+    <row r="52">
+      <c r="A52" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>h11</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C52" s="13" t="inlineStr">
         <is>
           <t>0.16.0</t>
         </is>
       </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="D52" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr">
         <is>
           <t>uvicorn</t>
         </is>
       </c>
-      <c r="F51" s="13" t="inlineStr">
+      <c r="F52" s="13" t="inlineStr">
         <is>
           <t>HTTP/1.1 protocol parser</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="n">
+    <row r="53">
+      <c r="A53" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>httpcore</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>1.0.9</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>BSD-3</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>httpx</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>Low-level HTTP transport</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="13" t="n">
+    <row r="54">
+      <c r="A54" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B53" s="13" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>idna</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C54" s="13" t="inlineStr">
         <is>
           <t>3.11</t>
         </is>
       </c>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="D54" s="13" t="inlineStr">
         <is>
           <t>BSD-3</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E54" s="13" t="inlineStr">
         <is>
           <t>requests</t>
         </is>
       </c>
-      <c r="F53" s="13" t="inlineStr">
+      <c r="F54" s="13" t="inlineStr">
         <is>
           <t>International domain names</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="n">
+    <row r="55">
+      <c r="A55" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>jaraco.classes</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>3.4.0</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>keyring</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>Class utilities</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="13" t="n">
+    <row r="56">
+      <c r="A56" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>jiter</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C56" s="13" t="inlineStr">
         <is>
           <t>0.13.0</t>
         </is>
       </c>
-      <c r="D55" s="13" t="inlineStr">
+      <c r="D56" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="E56" s="13" t="inlineStr">
         <is>
           <t>pydantic</t>
         </is>
       </c>
-      <c r="F55" s="13" t="inlineStr">
+      <c r="F56" s="13" t="inlineStr">
         <is>
           <t>Fast JSON parsing (Rust)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="n">
+    <row r="57">
+      <c r="A57" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>markdown-it-py</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>4.0.0</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>rich</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>Markdown parsing</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="13" t="n">
+    <row r="58">
+      <c r="A58" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>mdurl</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="D57" s="13" t="inlineStr">
+      <c r="D58" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E57" s="13" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>markdown-it-py</t>
         </is>
       </c>
-      <c r="F57" s="13" t="inlineStr">
+      <c r="F58" s="13" t="inlineStr">
         <is>
           <t>URL parsing for markdown</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="n">
+    <row r="59">
+      <c r="A59" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>more-itertools</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>10.8.0</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>keyring</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>Iterator utilities</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="13" t="n">
+    <row r="60">
+      <c r="A60" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>packaging</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C60" s="13" t="inlineStr">
         <is>
           <t>26.0</t>
         </is>
       </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="D60" s="13" t="inlineStr">
         <is>
           <t>Apache 2.0</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
+      <c r="E60" s="13" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="F59" s="13" t="inlineStr">
+      <c r="F60" s="13" t="inlineStr">
         <is>
           <t>Version parsing</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="4" t="n">
+    <row r="61">
+      <c r="A61" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>pycparser</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>BSD-3</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>cffi</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>C parser for FFI</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="13" t="n">
+    <row r="62">
+      <c r="A62" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="B61" s="13" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>pydantic_core</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>2.33.0</t>
         </is>
       </c>
-      <c r="D61" s="13" t="inlineStr">
+      <c r="D62" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E61" s="13" t="inlineStr">
+      <c r="E62" s="13" t="inlineStr">
         <is>
           <t>pydantic</t>
         </is>
       </c>
-      <c r="F61" s="13" t="inlineStr">
+      <c r="F62" s="13" t="inlineStr">
         <is>
           <t>Core validation engine (Rust)</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="4" t="n">
+    <row r="63">
+      <c r="A63" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>Pygments</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>2.19.2</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>BSD-2</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>rich</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>Syntax highlighting</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="13" t="n">
+    <row r="64">
+      <c r="A64" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>pywin32-ctypes</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C64" s="13" t="inlineStr">
         <is>
           <t>0.2.3</t>
         </is>
       </c>
-      <c r="D63" s="13" t="inlineStr">
+      <c r="D64" s="13" t="inlineStr">
         <is>
           <t>BSD-3</t>
         </is>
       </c>
-      <c r="E63" s="13" t="inlineStr">
+      <c r="E64" s="13" t="inlineStr">
         <is>
           <t>keyring (Windows)</t>
         </is>
       </c>
-      <c r="F63" s="13" t="inlineStr">
+      <c r="F64" s="13" t="inlineStr">
         <is>
           <t>Windows API access</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="4" t="n">
+    <row r="65">
+      <c r="A65" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>sniffio</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>1.3.1</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>httpx</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>Async library detection</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="13" t="n">
+    <row r="66">
+      <c r="A66" s="13" t="n">
         <v>22</v>
       </c>
-      <c r="B65" s="13" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>typing_extensions</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>4.15.0</t>
         </is>
       </c>
-      <c r="D65" s="13" t="inlineStr">
+      <c r="D66" s="13" t="inlineStr">
         <is>
           <t>PSF-2.0</t>
         </is>
       </c>
-      <c r="E65" s="13" t="inlineStr">
+      <c r="E66" s="13" t="inlineStr">
         <is>
           <t>pydantic</t>
         </is>
       </c>
-      <c r="F65" s="13" t="inlineStr">
+      <c r="F66" s="13" t="inlineStr">
         <is>
           <t>Python typing backports</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="4" t="n">
+    <row r="67">
+      <c r="A67" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>typing-inspection</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>0.4.2</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>pydantic</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>Type introspection</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="13" t="n">
+    <row r="68">
+      <c r="A68" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="B67" s="13" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>iniconfig</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C68" s="13" t="inlineStr">
         <is>
           <t>2.3.0</t>
         </is>
       </c>
-      <c r="D67" s="13" t="inlineStr">
+      <c r="D68" s="13" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E67" s="13" t="inlineStr">
+      <c r="E68" s="13" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="F67" s="13" t="inlineStr">
+      <c r="F68" s="13" t="inlineStr">
         <is>
           <t>INI file parsing for pytest config</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="n">
+    <row r="69">
+      <c r="A69" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>pluggy</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>1.6.0</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>Plugin framework for pytest</t>
         </is>
@@ -3625,7 +3670,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>